<commit_message>
iir filter file added
don't know others
</commit_message>
<xml_diff>
--- a/xlsx/5x5_data_blocks_with_gaps.xlsx
+++ b/xlsx/5x5_data_blocks_with_gaps.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,19 +418,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="B1" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="C1" t="n">
         <v>0</v>
       </c>
       <c r="D1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E1" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2">
@@ -441,18 +441,18 @@
         <v>-1</v>
       </c>
       <c r="C2" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E2" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="B3" t="n">
         <v>0</v>
@@ -461,44 +461,44 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D4" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="C5" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E5" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -510,16 +510,16 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="B7" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="C7" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
@@ -530,10 +530,10 @@
         <v>1</v>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="D8" t="n">
         <v>-1</v>
@@ -547,7 +547,7 @@
         <v>-1</v>
       </c>
       <c r="B9" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
         <v>1</v>
@@ -556,12 +556,12 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="n">
         <v>1</v>
@@ -573,24 +573,24 @@
         <v>-1</v>
       </c>
       <c r="E10" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="B11" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -602,7 +602,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="B13" t="n">
         <v>1</v>
@@ -611,10 +611,10 @@
         <v>-2</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="14">
@@ -628,44 +628,44 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
         <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D16" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="17">
@@ -673,16 +673,16 @@
         <v>-2</v>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D17" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -694,19 +694,19 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="D19" t="n">
         <v>-1</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="20">
@@ -717,10 +717,10 @@
         <v>-2</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="D20" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
@@ -740,7 +740,7 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -748,30 +748,30 @@
         <v>1</v>
       </c>
       <c r="B22" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="D22" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="D23" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -786,44 +786,44 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="B25" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="D25" t="n">
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
         <v>-2</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="B27" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
         <v>3</v>
@@ -832,24 +832,24 @@
         <v>-2</v>
       </c>
       <c r="E27" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="B28" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="29">
@@ -863,7 +863,7 @@
         <v>-1</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E29" t="n">
         <v>-1</v>
@@ -878,33 +878,33 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="E31" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="B32" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
@@ -912,53 +912,53 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C33" t="n">
         <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E33" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
         <v>-2</v>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="B35" t="n">
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D35" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -970,64 +970,64 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="B37" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D37" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="E37" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="B38" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="C38" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
         <v>-2</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="C39" t="n">
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="B40" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -1038,19 +1038,19 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="B41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C41" t="n">
         <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">

</xml_diff>